<commit_message>
Refactor master imports to add carline and remove unused fields
Added 'carline' field to MasterShikake and MasterCircuit models and imports. Removed 'issue', 'barcode_kanban', and 'released_note' fields from models, configs, and import logic. Updated template configs and import header validation to match new column structure. Adjusted migration files to add 'carline' and remove deprecated columns from master tables. Updated related Excel templates and adjusted column indices in importers.
</commit_message>
<xml_diff>
--- a/public/docs/Template_Cutting.xlsx
+++ b/public/docs/Template_Cutting.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\laragon\www\jai_ekanban\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44DE4BA4-C1D3-4661-99DA-DA067F559D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9541C229-A7A5-4FE5-B039-A7F29D9CCEB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{DB888F35-DBDA-4F92-8C17-F796FD33FFBE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Conveyor</t>
   </si>
@@ -50,21 +50,12 @@
     <t>Qty.</t>
   </si>
   <si>
-    <t>Issue</t>
-  </si>
-  <si>
     <t>Machine</t>
   </si>
   <si>
     <t>Sequence</t>
   </si>
   <si>
-    <t>Barcode Kanban</t>
-  </si>
-  <si>
-    <t>Released Date</t>
-  </si>
-  <si>
     <t>Released Note</t>
   </si>
   <si>
@@ -183,6 +174,9 @@
   </si>
   <si>
     <t>ASSY5</t>
+  </si>
+  <si>
+    <t>Carline</t>
   </si>
 </sst>
 </file>
@@ -286,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -302,6 +296,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -636,196 +633,188 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A02A7C30-A8FE-4581-AC4A-4E3166DD3C21}">
-  <dimension ref="A1:AW1"/>
+  <dimension ref="A1:AU1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="7.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="4.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="43" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="5.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="45" max="16384" width="9.140625" style="1"/>
+    <col min="8" max="8" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="4.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="41" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="5.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="43" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:47" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AI1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="3" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="3" t="s">
+      <c r="AK1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="3" t="s">
+      <c r="AL1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="3" t="s">
+      <c r="AM1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AN1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AO1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="3" t="s">
+      <c r="AP1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="3" t="s">
+      <c r="AQ1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="3" t="s">
+      <c r="AR1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="5" t="s">
+      <c r="AS1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="4" t="s">
+      <c r="AT1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="4" t="s">
+      <c r="AU1" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="AU1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="AV1" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="AW1" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add shikake_code, qrcode_shikake, master carline, UI improvements
- Add shikake_code field to master_circuit and qrcode_shikake to assy_schedule_circuit
- Generate qrcode_shikake in KanbanGeneratorService alongside barcode_kanban
- Add QRCODE SHIKAKE to CUTTING and TWIST print templates
- Rename all 'BARCODE KANBAN' labels to 'QRCODE KANBAN' across 8+ templates
- Add Master Carline module (model, service, controller, views, migration, menu)
- Add carline_id foreign key to master_family table
- Add circuit edit modal and upload drawing modal
- Split shikake detail/edit into separate view/edit modals
- Separate print preview (GET) from mark-as-printed (POST) for circuit and shikake
- Update CircuitTemplateConfig with Shikake Code column (index 19)
- Regenerate Template_Cutting.xlsx with new column
- Improve delete confirmations with detailed info display
- Update sidebar menu structure and MenuSeeder
</commit_message>
<xml_diff>
--- a/public/docs/Template_Cutting.xlsx
+++ b/public/docs/Template_Cutting.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="54">
   <si>
     <t>Type</t>
   </si>
@@ -74,6 +74,9 @@
     <t>CCT Code</t>
   </si>
   <si>
+    <t>Shikake Code</t>
+  </si>
+  <si>
     <t>Kind</t>
   </si>
   <si>
@@ -164,7 +167,7 @@
     <t>T06</t>
   </si>
   <si>
-    <t>MEMORI TWIST</t>
+    <t>Memory Twist</t>
   </si>
   <si>
     <t>ASSY-001</t>
@@ -564,7 +567,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:BA1"/>
+  <dimension ref="A1:BB1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="8.141" bestFit="true" customWidth="true" style="0"/>
@@ -586,43 +589,44 @@
     <col min="17" max="17" width="12.854" bestFit="true" customWidth="true" style="0"/>
     <col min="18" max="18" width="11.569" bestFit="true" customWidth="true" style="0"/>
     <col min="19" max="19" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="20" max="20" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="20" max="20" width="17.567" bestFit="true" customWidth="true" style="0"/>
     <col min="21" max="21" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="22" max="22" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="22" max="22" width="8.141" bestFit="true" customWidth="true" style="0"/>
     <col min="23" max="23" width="6.856" bestFit="true" customWidth="true" style="0"/>
-    <col min="24" max="24" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="25" max="25" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="24" max="24" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="25" max="25" width="15.139" bestFit="true" customWidth="true" style="0"/>
     <col min="26" max="26" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="27" max="27" width="11.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="28" max="28" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="29" max="29" width="11.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="30" max="30" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="27" max="27" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="28" max="28" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="29" max="29" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="30" max="30" width="11.569" bestFit="true" customWidth="true" style="0"/>
     <col min="31" max="31" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="32" max="32" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="33" max="33" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="34" max="34" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="32" max="32" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="33" max="33" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="34" max="34" width="15.139" bestFit="true" customWidth="true" style="0"/>
     <col min="35" max="35" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="36" max="36" width="11.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="37" max="37" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="38" max="38" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="36" max="36" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="37" max="37" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="38" max="38" width="9.283" bestFit="true" customWidth="true" style="0"/>
     <col min="39" max="39" width="10.426" bestFit="true" customWidth="true" style="0"/>
     <col min="40" max="40" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="41" max="41" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="42" max="42" width="5.713" bestFit="true" customWidth="true" style="0"/>
+    <col min="41" max="41" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="42" max="42" width="12.854" bestFit="true" customWidth="true" style="0"/>
     <col min="43" max="43" width="5.713" bestFit="true" customWidth="true" style="0"/>
-    <col min="44" max="44" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="44" max="44" width="5.713" bestFit="true" customWidth="true" style="0"/>
     <col min="45" max="45" width="6.856" bestFit="true" customWidth="true" style="0"/>
     <col min="46" max="46" width="6.856" bestFit="true" customWidth="true" style="0"/>
     <col min="47" max="47" width="6.856" bestFit="true" customWidth="true" style="0"/>
     <col min="48" max="48" width="6.856" bestFit="true" customWidth="true" style="0"/>
     <col min="49" max="49" width="6.856" bestFit="true" customWidth="true" style="0"/>
-    <col min="50" max="50" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="51" max="51" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="50" max="50" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="51" max="51" width="17.567" bestFit="true" customWidth="true" style="0"/>
     <col min="52" max="52" width="12.854" bestFit="true" customWidth="true" style="0"/>
     <col min="53" max="53" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="54" max="54" width="12.854" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:53">
+    <row r="1" spans="1:54">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -773,7 +777,7 @@
       <c r="AX1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="AZ1" s="2" t="s">
@@ -781,6 +785,9 @@
       </c>
       <c r="BA1" s="2" t="s">
         <v>52</v>
+      </c>
+      <c r="BB1" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: add barcode_twist & qrcode_drawing to circuit print, template, and edit/view modals
- EkanbanCircuitService: add barcode_twist & qrcode_drawing to getCircuitsForPrint() SELECT query so barcode/QR images are generated correctly on print preview and QZ Tray
- Template_Cutting.xlsx: regenerate template to include Barcode Twist (col Q) and QRCode Drawing (col R)
- detail_modal: add Barcode Twist and QRCode Drawing rows to view modal
- edit_modal: add Barcode section (barcode_mesin, barcode_navigasi, barcode_process, barcode_shikake) as full-width form fields
- index.blade.php: populate barcode_twist, qrcode_drawing in view handler and all 4 barcode fields in edit handler
</commit_message>
<xml_diff>
--- a/public/docs/Template_Cutting.xlsx
+++ b/public/docs/Template_Cutting.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
   <si>
     <t>Type</t>
   </si>
@@ -63,6 +63,12 @@
   </si>
   <si>
     <t>Barcode Shikake</t>
+  </si>
+  <si>
+    <t>Barcode Twist</t>
+  </si>
+  <si>
+    <t>QRCode Drawing</t>
   </si>
   <si>
     <t>To Store</t>
@@ -567,7 +573,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:BB1"/>
+  <dimension ref="A1:BD1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="8.141" bestFit="true" customWidth="true" style="0"/>
@@ -586,47 +592,49 @@
     <col min="14" max="14" width="22.28" bestFit="true" customWidth="true" style="0"/>
     <col min="15" max="15" width="20.995" bestFit="true" customWidth="true" style="0"/>
     <col min="16" max="16" width="20.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="17" max="17" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="18" max="18" width="19.852" bestFit="true" customWidth="true" style="0"/>
     <col min="19" max="19" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="20" max="20" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="21" max="21" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="22" max="22" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="23" max="23" width="6.856" bestFit="true" customWidth="true" style="0"/>
-    <col min="24" max="24" width="6.856" bestFit="true" customWidth="true" style="0"/>
-    <col min="25" max="25" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="26" max="26" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="27" max="27" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="28" max="28" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="20" max="20" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="21" max="21" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="22" max="22" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="23" max="23" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="24" max="24" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="25" max="25" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="26" max="26" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="27" max="27" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="28" max="28" width="10.426" bestFit="true" customWidth="true" style="0"/>
     <col min="29" max="29" width="10.426" bestFit="true" customWidth="true" style="0"/>
     <col min="30" max="30" width="11.569" bestFit="true" customWidth="true" style="0"/>
     <col min="31" max="31" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="32" max="32" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="33" max="33" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="34" max="34" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="35" max="35" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="36" max="36" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="37" max="37" width="11.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="38" max="38" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="39" max="39" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="40" max="40" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="32" max="32" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="33" max="33" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="34" max="34" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="35" max="35" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="36" max="36" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="37" max="37" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="38" max="38" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="39" max="39" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="40" max="40" width="9.283" bestFit="true" customWidth="true" style="0"/>
     <col min="41" max="41" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="42" max="42" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="43" max="43" width="5.713" bestFit="true" customWidth="true" style="0"/>
-    <col min="44" max="44" width="5.713" bestFit="true" customWidth="true" style="0"/>
-    <col min="45" max="45" width="6.856" bestFit="true" customWidth="true" style="0"/>
-    <col min="46" max="46" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="42" max="42" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="43" max="43" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="44" max="44" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="45" max="45" width="5.713" bestFit="true" customWidth="true" style="0"/>
+    <col min="46" max="46" width="5.713" bestFit="true" customWidth="true" style="0"/>
     <col min="47" max="47" width="6.856" bestFit="true" customWidth="true" style="0"/>
     <col min="48" max="48" width="6.856" bestFit="true" customWidth="true" style="0"/>
     <col min="49" max="49" width="6.856" bestFit="true" customWidth="true" style="0"/>
     <col min="50" max="50" width="6.856" bestFit="true" customWidth="true" style="0"/>
-    <col min="51" max="51" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="52" max="52" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="53" max="53" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="51" max="51" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="52" max="52" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="53" max="53" width="17.567" bestFit="true" customWidth="true" style="0"/>
     <col min="54" max="54" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="55" max="55" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="56" max="56" width="12.854" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54">
+    <row r="1" spans="1:56">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -780,14 +788,20 @@
       <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
       <c r="BB1" s="2" t="s">
         <v>53</v>
+      </c>
+      <c r="BC1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD1" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>